<commit_message>
Create R script for surface coverage and bleaching
</commit_message>
<xml_diff>
--- a/data/daily_measurements.xlsx
+++ b/data/daily_measurements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruben/dev/duckweed-rmbe/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13D0D180-6A0D-B141-A771-F20349C3FCF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA500D6-680D-0549-9E77-AF8CBEEFB068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="980" yWindow="1260" windowWidth="27840" windowHeight="16240" xr2:uid="{1AF4B679-1F14-8444-99BB-B7E1E6DBFAB9}"/>
   </bookViews>
@@ -457,6 +457,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BBE42C9-4347-6048-B2F8-34461A0CE087}">
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -605,7 +608,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="2">
-        <v>46181.693055555559</v>
+        <v>46182.688888888886</v>
       </c>
       <c r="G6" s="1">
         <v>35.68</v>
@@ -631,7 +634,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="2">
-        <v>46181.693055555559</v>
+        <v>46182.688888888886</v>
       </c>
       <c r="G7" s="1">
         <v>30.27</v>
@@ -657,7 +660,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="2">
-        <v>46181.693055555559</v>
+        <v>46182.688888888886</v>
       </c>
       <c r="G8" s="1">
         <v>38.270000000000003</v>
@@ -683,7 +686,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="2">
-        <v>46181.693055555559</v>
+        <v>46182.688888888886</v>
       </c>
       <c r="G9" s="1">
         <v>53.24</v>
@@ -694,5 +697,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Measurements day 3 and 4
</commit_message>
<xml_diff>
--- a/data/daily_measurements.xlsx
+++ b/data/daily_measurements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruben/dev/duckweed-rmbe/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEDD8AE-0B8E-0241-9401-41950F5BF0EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ABCE29E-3D5A-764D-ACF9-401B3969515D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14700" yWindow="760" windowWidth="14700" windowHeight="16740" xr2:uid="{1AF4B679-1F14-8444-99BB-B7E1E6DBFAB9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="12">
   <si>
     <t>container_id</t>
   </si>
@@ -455,10 +455,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BBE42C9-4347-6048-B2F8-34461A0CE087}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -796,6 +802,214 @@
         <v>64.23</v>
       </c>
       <c r="H13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>3</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G14" s="1">
+        <v>73.069999999999993</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>4</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G15" s="1">
+        <v>70.08</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>7</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G16" s="1">
+        <v>64.150000000000006</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>8</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G17" s="1">
+        <v>74.78</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>3</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G18" s="1">
+        <v>54.62</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>4</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="1">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G19" s="1">
+        <v>72.680000000000007</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>7</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G20" s="1">
+        <v>70.08</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>8</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>4</v>
+      </c>
+      <c r="F21" s="2">
+        <v>46183.601388888892</v>
+      </c>
+      <c r="G21" s="1">
+        <v>73.5</v>
+      </c>
+      <c r="H21" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix measurements day 4
</commit_message>
<xml_diff>
--- a/data/daily_measurements.xlsx
+++ b/data/daily_measurements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruben/dev/duckweed-rmbe/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ABCE29E-3D5A-764D-ACF9-401B3969515D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F972452-B9B8-3B48-A7D0-39EB9EA28929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14700" yWindow="760" windowWidth="14700" windowHeight="16740" xr2:uid="{1AF4B679-1F14-8444-99BB-B7E1E6DBFAB9}"/>
   </bookViews>
@@ -929,7 +929,7 @@
         <v>46183.601388888892</v>
       </c>
       <c r="G18" s="1">
-        <v>54.62</v>
+        <v>79.180000000000007</v>
       </c>
       <c r="H18" s="1">
         <v>0</v>
@@ -955,7 +955,7 @@
         <v>46183.601388888892</v>
       </c>
       <c r="G19" s="1">
-        <v>72.680000000000007</v>
+        <v>81.98</v>
       </c>
       <c r="H19" s="1">
         <v>0</v>
@@ -981,7 +981,7 @@
         <v>46183.601388888892</v>
       </c>
       <c r="G20" s="1">
-        <v>70.08</v>
+        <v>89.41</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -1007,7 +1007,7 @@
         <v>46183.601388888892</v>
       </c>
       <c r="G21" s="1">
-        <v>73.5</v>
+        <v>81.36</v>
       </c>
       <c r="H21" s="1">
         <v>0</v>

</xml_diff>